<commit_message>
update font on every pages
</commit_message>
<xml_diff>
--- a/data/lessons.xlsx
+++ b/data/lessons.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Data/Work/Education/learning-hub/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5ECE75F-0ECE-2D4F-B405-FE33FBE78281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA0B0E4-724A-7348-898E-0624BBA585E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16660" activeTab="3" xr2:uid="{1E661350-D387-A54E-832B-3163FAE13FCA}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="77">
   <si>
     <t>id</t>
   </si>
@@ -113,30 +113,12 @@
     <t>audio</t>
   </si>
   <si>
-    <t>小明早上起床。</t>
-  </si>
-  <si>
-    <t>Xiǎomíng zǎoshang qǐchuáng.</t>
-  </si>
-  <si>
-    <t>Xiaoming gets up in the morning.</t>
-  </si>
-  <si>
     <t>assets/images/story-01.jpg</t>
   </si>
   <si>
     <t>assets/audio/story-01.mp3</t>
   </si>
   <si>
-    <t>他去学校。</t>
-  </si>
-  <si>
-    <t>Tā qù xuéxiào.</t>
-  </si>
-  <si>
-    <t>He goes to school.</t>
-  </si>
-  <si>
     <t>assets/images/story-02.jpg</t>
   </si>
   <si>
@@ -188,19 +170,109 @@
     <t>multiple-choice</t>
   </si>
   <si>
-    <t>What does 学校 mean?</t>
-  </si>
-  <si>
-    <t>School</t>
-  </si>
-  <si>
-    <t>Teacher</t>
-  </si>
-  <si>
-    <t>Friend</t>
-  </si>
-  <si>
-    <t>Morning</t>
+    <t>早上好！</t>
+  </si>
+  <si>
+    <t>Zǎoshang hǎo!</t>
+  </si>
+  <si>
+    <t>Good morning!</t>
+  </si>
+  <si>
+    <t>小明起床了。</t>
+  </si>
+  <si>
+    <t>Xiǎomíng qǐchuáng le.</t>
+  </si>
+  <si>
+    <t>Xiaoming gets up.</t>
+  </si>
+  <si>
+    <t>他吃早饭。</t>
+  </si>
+  <si>
+    <t>Tā chī zǎofàn.</t>
+  </si>
+  <si>
+    <t>He eats breakfast.</t>
+  </si>
+  <si>
+    <t>assets/images/story-03.jpg</t>
+  </si>
+  <si>
+    <t>assets/audio/story-03.mp3</t>
+  </si>
+  <si>
+    <t>然后，他去学校。</t>
+  </si>
+  <si>
+    <t>Ránhòu, tā qù xuéxiào.</t>
+  </si>
+  <si>
+    <t>Then, he goes to school.</t>
+  </si>
+  <si>
+    <t>assets/images/story-04.jpg</t>
+  </si>
+  <si>
+    <t>assets/audio/story-04.mp3</t>
+  </si>
+  <si>
+    <t>他很开心。</t>
+  </si>
+  <si>
+    <t>Tā hěn kāixīn.</t>
+  </si>
+  <si>
+    <t>He is very happy.</t>
+  </si>
+  <si>
+    <t>assets/images/story-05.jpg</t>
+  </si>
+  <si>
+    <t>assets/audio/story-05.mp3</t>
+  </si>
+  <si>
+    <t>assets/audio/zaoshang.mp3</t>
+  </si>
+  <si>
+    <t>起床</t>
+  </si>
+  <si>
+    <t>qǐchuáng</t>
+  </si>
+  <si>
+    <t>get up</t>
+  </si>
+  <si>
+    <t>assets/audio/qichuang.mp3</t>
+  </si>
+  <si>
+    <t>assets/audio/xuexiao.mp3</t>
+  </si>
+  <si>
+    <t>开心</t>
+  </si>
+  <si>
+    <t>kāixīn</t>
+  </si>
+  <si>
+    <t>happy</t>
+  </si>
+  <si>
+    <t>assets/audio/kaixin.mp3</t>
+  </si>
+  <si>
+    <t>Where does Xiaoming go?</t>
+  </si>
+  <si>
+    <t>家 — Home</t>
+  </si>
+  <si>
+    <t>学校 — School</t>
+  </si>
+  <si>
+    <t>商店 — Shop</t>
   </si>
 </sst>
 </file>
@@ -649,7 +721,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F654DC2-C5DD-1D44-89B9-36C308A6DA2B}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -683,19 +755,19 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>24</v>
-      </c>
-      <c r="E2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -706,19 +778,88 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -728,7 +869,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8662A019-9790-E945-AE9A-5DE776F254B5}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -739,7 +880,7 @@
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -759,13 +900,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -776,13 +920,56 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="E3" t="s">
-        <v>39</v>
+        <v>66</v>
+      </c>
+      <c r="F3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -803,25 +990,25 @@
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -832,25 +1019,22 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="F2" t="s">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H2" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="I2" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add full audio support and audio feedback
- Add `fullAudio` path to lesson data and UI
- Implement audio feedback sounds for exercises
- Refactor tone playback to prevent auto-play on load
</commit_message>
<xml_diff>
--- a/data/lessons.xlsx
+++ b/data/lessons.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -431,6 +431,9 @@
       <c r="I1" t="str">
         <v>poster</v>
       </c>
+      <c r="J1" t="str">
+        <v>fullAudio</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -460,6 +463,9 @@
       <c r="I2" t="str">
         <v>assets/images/story-poster.jpg</v>
       </c>
+      <c r="J2" t="str">
+        <v>assets/audio/lesson-01-full.mp3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -489,10 +495,13 @@
       <c r="I3" t="str">
         <v>assets/images/story2-poster.jpg</v>
       </c>
+      <c r="J3" t="str">
+        <v>assets/audio/lesson-02-full.mp3</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1107,7 +1116,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:K11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1141,9 +1150,6 @@
         <v>optionC</v>
       </c>
       <c r="K1" t="str">
-        <v>optionD</v>
-      </c>
-      <c r="L1" t="str">
         <v>answer</v>
       </c>
     </row>
@@ -1243,6 +1249,9 @@
       <c r="E6" t="str">
         <v>question particle</v>
       </c>
+      <c r="F6" t="str">
+        <v>assets/audio/tones/ma-tone-5.mp3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1303,7 +1312,7 @@
       <c r="J9" t="str">
         <v>再见</v>
       </c>
-      <c r="L9" t="str">
+      <c r="K9" t="str">
         <v>你好</v>
       </c>
     </row>
@@ -1326,7 +1335,7 @@
       <c r="J10" t="str">
         <v>Where are you?</v>
       </c>
-      <c r="L10" t="str">
+      <c r="K10" t="str">
         <v>How are you?</v>
       </c>
     </row>
@@ -1351,9 +1360,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add lesson search and keyword filtering
Implemented a search bar and topic filter chips to allow users to easily find lessons by keywords, pinyin, or Chinese. Added metadata keywords to existing lessons to support the new search functionality.
</commit_message>
<xml_diff>
--- a/data/lessons.xlsx
+++ b/data/lessons.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,6 +434,9 @@
       <c r="J1" t="str">
         <v>fullAudio</v>
       </c>
+      <c r="K1" t="str">
+        <v>keywords</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -466,6 +469,9 @@
       <c r="J2" t="str">
         <v>assets/audio/lesson-01-full.mp3</v>
       </c>
+      <c r="K2" t="str">
+        <v>morning, routine, breakfast, school, happy, day, get up, early, 早上, 起床, 学校, 早饭, 开心</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -498,10 +504,13 @@
       <c r="J3" t="str">
         <v>assets/audio/lesson-02-full.mp3</v>
       </c>
+      <c r="K3" t="str">
+        <v>fruit, market, apple, shopping, fresh, sweet, delicious, red, buy, 水果, 市场, 苹果, 买, 甜, 好吃</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add interactive learning games module
- Include new "Games" sheet in data structure
- Implement games.html and games-embed.html for game content delivery
- Add new hero banner and Wordwall game integrations to learning hub
</commit_message>
<xml_diff>
--- a/data/lessons.xlsx
+++ b/data/lessons.xlsx
@@ -8,6 +8,7 @@
     <sheet name="Vocabulary" sheetId="3" r:id="rId3"/>
     <sheet name="Exercises" sheetId="4" r:id="rId4"/>
     <sheet name="Demo" sheetId="5" r:id="rId5"/>
+    <sheet name="Games" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -1373,4 +1374,120 @@
     <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>order</v>
+      </c>
+      <c r="C1" t="str">
+        <v>title</v>
+      </c>
+      <c r="D1" t="str">
+        <v>category</v>
+      </c>
+      <c r="E1" t="str">
+        <v>badge</v>
+      </c>
+      <c r="F1" t="str">
+        <v>description</v>
+      </c>
+      <c r="G1" t="str">
+        <v>embed_code</v>
+      </c>
+      <c r="H1" t="str">
+        <v>embed_url</v>
+      </c>
+      <c r="I1" t="str">
+        <v>width</v>
+      </c>
+      <c r="J1" t="str">
+        <v>height</v>
+      </c>
+      <c r="K1" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>game-01</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Tone Hunter — Character &amp; Tone Matcher</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Tone Recognition</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Wordwall Challenge 1</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Match Mandarin characters to their correct tone mark and phonetic pitch. Practice tonal accuracy and ear training.</v>
+      </c>
+      <c r="G2" t="str">
+        <v>&lt;iframe style="max-width:100%" src="https://wordwall.net/embed/9dfb097b6b4a405ca39a08514e805030?themeId=27&amp;templateId=82&amp;fontStackId=0" width="500" height="380" frameborder="0" allowfullscreen&gt;&lt;/iframe&gt;</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://wordwall.net/embed/9dfb097b6b4a405ca39a08514e805030?themeId=27&amp;templateId=82&amp;fontStackId=0</v>
+      </c>
+      <c r="I2">
+        <v>500</v>
+      </c>
+      <c r="J2">
+        <v>380</v>
+      </c>
+      <c r="K2" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>game-02</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Word Speed Quiz — Vocabulary Match</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Rapid Recall</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Wordwall Challenge 2</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Fast-paced Mandarin vocabulary identification. Test your speed recognition of characters, pinyin, and definitions.</v>
+      </c>
+      <c r="G3" t="str">
+        <v>&lt;iframe style="max-width:100%" src="https://wordwall.net/embed/9dfb097b6b4a405ca39a08514e805030?themeId=23&amp;templateId=49&amp;fontStackId=0" width="500" height="380" frameborder="0" allowfullscreen&gt;&lt;/iframe&gt;</v>
+      </c>
+      <c r="H3" t="str">
+        <v>https://wordwall.net/embed/9dfb097b6b4a405ca39a08514e805030?themeId=23&amp;templateId=49&amp;fontStackId=0</v>
+      </c>
+      <c r="I3">
+        <v>500</v>
+      </c>
+      <c r="J3">
+        <v>380</v>
+      </c>
+      <c r="K3" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: remove demo section from lessons
Delete the "Demo" lesson sheet and associated UI code, styling, and data processing logic to simplify the codebase.
</commit_message>
<xml_diff>
--- a/data/lessons.xlsx
+++ b/data/lessons.xlsx
@@ -7,8 +7,7 @@
     <sheet name="Story" sheetId="2" r:id="rId2"/>
     <sheet name="Vocabulary" sheetId="3" r:id="rId3"/>
     <sheet name="Exercises" sheetId="4" r:id="rId4"/>
-    <sheet name="Demo" sheetId="5" r:id="rId5"/>
-    <sheet name="Games" sheetId="6" r:id="rId6"/>
+    <sheet name="Games" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -1126,258 +1125,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K11"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>section</v>
-      </c>
-      <c r="B1" t="str">
-        <v>order</v>
-      </c>
-      <c r="C1" t="str">
-        <v>chinese</v>
-      </c>
-      <c r="D1" t="str">
-        <v>pinyin</v>
-      </c>
-      <c r="E1" t="str">
-        <v>english</v>
-      </c>
-      <c r="F1" t="str">
-        <v>audio</v>
-      </c>
-      <c r="G1" t="str">
-        <v>question</v>
-      </c>
-      <c r="H1" t="str">
-        <v>optionA</v>
-      </c>
-      <c r="I1" t="str">
-        <v>optionB</v>
-      </c>
-      <c r="J1" t="str">
-        <v>optionC</v>
-      </c>
-      <c r="K1" t="str">
-        <v>answer</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Pronunciation</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="str">
-        <v>妈</v>
-      </c>
-      <c r="D2" t="str">
-        <v>mā</v>
-      </c>
-      <c r="E2" t="str">
-        <v>mother</v>
-      </c>
-      <c r="F2" t="str">
-        <v>assets/audio/tones/ma-tone-1.mp3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Pronunciation</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" t="str">
-        <v>麻</v>
-      </c>
-      <c r="D3" t="str">
-        <v>má</v>
-      </c>
-      <c r="E3" t="str">
-        <v>hemp; numb</v>
-      </c>
-      <c r="F3" t="str">
-        <v>assets/audio/tones/ma-tone-2.mp3</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Pronunciation</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4" t="str">
-        <v>马</v>
-      </c>
-      <c r="D4" t="str">
-        <v>mǎ</v>
-      </c>
-      <c r="E4" t="str">
-        <v>horse</v>
-      </c>
-      <c r="F4" t="str">
-        <v>assets/audio/tones/ma-tone-3.mp3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Pronunciation</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5" t="str">
-        <v>骂</v>
-      </c>
-      <c r="D5" t="str">
-        <v>mà</v>
-      </c>
-      <c r="E5" t="str">
-        <v>scold</v>
-      </c>
-      <c r="F5" t="str">
-        <v>assets/audio/tones/ma-tone-4.mp3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Pronunciation</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6" t="str">
-        <v>吗</v>
-      </c>
-      <c r="D6" t="str">
-        <v>ma</v>
-      </c>
-      <c r="E6" t="str">
-        <v>question particle</v>
-      </c>
-      <c r="F6" t="str">
-        <v>assets/audio/tones/ma-tone-5.mp3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Everyday Chinese</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" t="str">
-        <v>你好</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Nǐ hǎo</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Hello</v>
-      </c>
-      <c r="F7" t="str">
-        <v>assets/audio/hello.mp3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Conversation</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="str">
-        <v>你好！你好吗？</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Nǐ hǎo! Nǐ hǎo ma?</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Hello! How are you?</v>
-      </c>
-      <c r="F8" t="str">
-        <v>assets/audio/nihao-conversation.mp3</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Quick Check</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="G9" t="str">
-        <v>How do you say “Hello” in Chinese?</v>
-      </c>
-      <c r="H9" t="str">
-        <v>你好</v>
-      </c>
-      <c r="I9" t="str">
-        <v>谢谢</v>
-      </c>
-      <c r="J9" t="str">
-        <v>再见</v>
-      </c>
-      <c r="K9" t="str">
-        <v>你好</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Quick Check</v>
-      </c>
-      <c r="B10">
-        <v>2</v>
-      </c>
-      <c r="G10" t="str">
-        <v>What does “你好吗？” mean?</v>
-      </c>
-      <c r="H10" t="str">
-        <v>What's your name?</v>
-      </c>
-      <c r="I10" t="str">
-        <v>How are you?</v>
-      </c>
-      <c r="J10" t="str">
-        <v>Where are you?</v>
-      </c>
-      <c r="K10" t="str">
-        <v>How are you?</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Conversation</v>
-      </c>
-      <c r="B11">
-        <v>2</v>
-      </c>
-      <c r="C11" t="str">
-        <v>早上好 !</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Zǎo Shang hǎo!</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Good Morning !</v>
-      </c>
-      <c r="F11" t="str">
-        <v>assets/audio/morning-conversation.mp3</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K3"/>
   <sheetData>
     <row r="1">

</xml_diff>